<commit_message>
updated with Brazil PR
</commit_message>
<xml_diff>
--- a/Brazil.xlsx
+++ b/Brazil.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\jaytanik\Documents\Feature_1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{788D40F9-B9DE-4A4E-BD9A-64780F18EA48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02CF46CD-649E-4273-85BB-F8D894069788}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="26160" windowHeight="16260" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -123,16 +123,16 @@
     <t>Freight In - Imports (52106)</t>
   </si>
   <si>
-    <t>Unspecified (0000)</t>
-  </si>
-  <si>
-    <t>Non-Designated Channel - Legacy (0000)</t>
-  </si>
-  <si>
-    <t>Unspecified 0000 (0000)</t>
-  </si>
-  <si>
     <t>Unit Price</t>
+  </si>
+  <si>
+    <t>Unspecified</t>
+  </si>
+  <si>
+    <t>Non-Designated Channel - Leg</t>
+  </si>
+  <si>
+    <t>Unspecified 0</t>
   </si>
 </sst>
 </file>
@@ -548,7 +548,7 @@
         <v>27</v>
       </c>
       <c r="W1" s="4" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2" spans="1:23" ht="105" x14ac:dyDescent="0.25">
@@ -601,19 +601,19 @@
         <v>0</v>
       </c>
       <c r="Q2" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="R2" s="3">
         <v>0</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="T2" s="3">
         <v>0</v>
       </c>
       <c r="U2" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="V2">
         <v>0</v>

</xml_diff>